<commit_message>
Added Scheduled Jobs For Scans
</commit_message>
<xml_diff>
--- a/Scanner/trading_toolkit.xlsx
+++ b/Scanner/trading_toolkit.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Risk-Reward Calculator" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="BSEGain_26Jul26" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="BSE1000_27Jul26" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="BSEGain_27Jul26" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -85022,4 +85023,1433 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" style="45" min="1" max="1"/>
+    <col width="26" customWidth="1" style="45" min="2" max="2"/>
+    <col width="15" customWidth="1" style="45" min="3" max="3"/>
+    <col width="15" customWidth="1" style="45" min="4" max="4"/>
+    <col width="15" customWidth="1" style="45" min="5" max="5"/>
+    <col width="15" customWidth="1" style="45" min="6" max="6"/>
+    <col width="15" customWidth="1" style="45" min="7" max="7"/>
+    <col width="15" customWidth="1" style="45" min="8" max="8"/>
+    <col width="15" customWidth="1" style="45" min="9" max="9"/>
+    <col width="15" customWidth="1" style="45" min="10" max="10"/>
+    <col width="15" customWidth="1" style="45" min="11" max="11"/>
+    <col width="15" customWidth="1" style="45" min="12" max="12"/>
+    <col width="15" customWidth="1" style="45" min="13" max="13"/>
+    <col width="15" customWidth="1" style="45" min="14" max="14"/>
+    <col width="15" customWidth="1" style="45" min="15" max="15"/>
+    <col width="15" customWidth="1" style="45" min="16" max="16"/>
+    <col width="15" customWidth="1" style="45" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="88" t="inlineStr">
+        <is>
+          <t>BSE Top Gainers (5.0%-20.0%) — 27 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="89" t="inlineStr">
+        <is>
+          <t>ALL BSE GAINERS 5.0%-20.0% — 11 stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1" s="45">
+      <c r="A4" s="90" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B4" s="90" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="90" t="inlineStr">
+        <is>
+          <t>Cap Segment</t>
+        </is>
+      </c>
+      <c r="D4" s="90" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="E4" s="90" t="inlineStr">
+        <is>
+          <t>% Chg</t>
+        </is>
+      </c>
+      <c r="F4" s="90" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="G4" s="90" t="inlineStr">
+        <is>
+          <t>Turnover (Rs Cr)</t>
+        </is>
+      </c>
+      <c r="H4" s="90" t="inlineStr">
+        <is>
+          <t>Vol Ratio (vs 3d avg)</t>
+        </is>
+      </c>
+      <c r="I4" s="90" t="inlineStr">
+        <is>
+          <t>Vol Ratio (vs 20d avg)</t>
+        </is>
+      </c>
+      <c r="J4" s="90" t="inlineStr">
+        <is>
+          <t>RSI(14)</t>
+        </is>
+      </c>
+      <c r="K4" s="90" t="inlineStr">
+        <is>
+          <t>ADX(14)</t>
+        </is>
+      </c>
+      <c r="L4" s="90" t="inlineStr">
+        <is>
+          <t>Score (0-9)</t>
+        </is>
+      </c>
+      <c r="M4" s="90" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="91" t="inlineStr">
+        <is>
+          <t>KFINTECH</t>
+        </is>
+      </c>
+      <c r="B5" s="91" t="inlineStr">
+        <is>
+          <t>KFin Technologies Limited</t>
+        </is>
+      </c>
+      <c r="C5" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D5" s="91" t="n">
+        <v>930.2</v>
+      </c>
+      <c r="E5" s="91" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="F5" s="91" t="n">
+        <v>4584202</v>
+      </c>
+      <c r="G5" s="91" t="n">
+        <v>426.42</v>
+      </c>
+      <c r="H5" s="91" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="I5" s="91" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J5" s="91" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="K5" s="91" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="L5" s="91" t="n">
+        <v>5</v>
+      </c>
+      <c r="M5" s="91" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="93" t="inlineStr">
+        <is>
+          <t>SAGILITY</t>
+        </is>
+      </c>
+      <c r="B6" s="93" t="inlineStr">
+        <is>
+          <t>Sagility Limited</t>
+        </is>
+      </c>
+      <c r="C6" s="93" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D6" s="93" t="n">
+        <v>43.37</v>
+      </c>
+      <c r="E6" s="93" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F6" s="93" t="n">
+        <v>65364693</v>
+      </c>
+      <c r="G6" s="93" t="n">
+        <v>283.49</v>
+      </c>
+      <c r="H6" s="93" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="I6" s="93" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="J6" s="93" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="K6" s="93" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="L6" s="93" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" s="93" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="91" t="inlineStr">
+        <is>
+          <t>REDINGTON</t>
+        </is>
+      </c>
+      <c r="B7" s="91" t="inlineStr">
+        <is>
+          <t>Redington Limited</t>
+        </is>
+      </c>
+      <c r="C7" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D7" s="91" t="n">
+        <v>277.8</v>
+      </c>
+      <c r="E7" s="91" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="F7" s="91" t="n">
+        <v>3947068</v>
+      </c>
+      <c r="G7" s="91" t="n">
+        <v>109.65</v>
+      </c>
+      <c r="H7" s="91" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="I7" s="91" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="J7" s="91" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="K7" s="91" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="L7" s="91" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="91" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="93" t="inlineStr">
+        <is>
+          <t>LATENTVIEW</t>
+        </is>
+      </c>
+      <c r="B8" s="93" t="inlineStr">
+        <is>
+          <t>Latent View Analytics Limited</t>
+        </is>
+      </c>
+      <c r="C8" s="93" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D8" s="93" t="n">
+        <v>316.3</v>
+      </c>
+      <c r="E8" s="93" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="F8" s="93" t="n">
+        <v>3557729</v>
+      </c>
+      <c r="G8" s="93" t="n">
+        <v>112.53</v>
+      </c>
+      <c r="H8" s="93" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="I8" s="93" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="J8" s="93" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="K8" s="93" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="L8" s="93" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" s="93" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="91" t="inlineStr">
+        <is>
+          <t>CAPLIPOINT</t>
+        </is>
+      </c>
+      <c r="B9" s="91" t="inlineStr">
+        <is>
+          <t>CAPLIN POINT LABORATORIES LTD.</t>
+        </is>
+      </c>
+      <c r="C9" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D9" s="91" t="n">
+        <v>2620.5</v>
+      </c>
+      <c r="E9" s="91" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="F9" s="91" t="n">
+        <v>241249</v>
+      </c>
+      <c r="G9" s="91" t="n">
+        <v>63.22</v>
+      </c>
+      <c r="H9" s="91" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="I9" s="91" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J9" s="91" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="K9" s="91" t="n">
+        <v>33</v>
+      </c>
+      <c r="L9" s="91" t="n">
+        <v>8</v>
+      </c>
+      <c r="M9" s="91" t="inlineStr">
+        <is>
+          <t>STRONG SETUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="93" t="inlineStr">
+        <is>
+          <t>LALPATHLAB</t>
+        </is>
+      </c>
+      <c r="B10" s="93" t="inlineStr">
+        <is>
+          <t>Dr. Lal Pathlabs Limited</t>
+        </is>
+      </c>
+      <c r="C10" s="93" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D10" s="93" t="n">
+        <v>1867.3</v>
+      </c>
+      <c r="E10" s="93" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="F10" s="93" t="n">
+        <v>1688883</v>
+      </c>
+      <c r="G10" s="93" t="n">
+        <v>315.37</v>
+      </c>
+      <c r="H10" s="93" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="I10" s="93" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="J10" s="93" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="K10" s="93" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="L10" s="93" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="93" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="91" t="inlineStr">
+        <is>
+          <t>ATUL</t>
+        </is>
+      </c>
+      <c r="B11" s="91" t="inlineStr">
+        <is>
+          <t>ATUL LTD.</t>
+        </is>
+      </c>
+      <c r="C11" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D11" s="91" t="n">
+        <v>6799.5</v>
+      </c>
+      <c r="E11" s="91" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="F11" s="91" t="n">
+        <v>239050</v>
+      </c>
+      <c r="G11" s="91" t="n">
+        <v>162.54</v>
+      </c>
+      <c r="H11" s="91" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="I11" s="91" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="J11" s="91" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="K11" s="91" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="L11" s="91" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="91" t="inlineStr">
+        <is>
+          <t>STRONG SETUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="93" t="inlineStr">
+        <is>
+          <t>TBOTEK</t>
+        </is>
+      </c>
+      <c r="B12" s="93" t="inlineStr">
+        <is>
+          <t>TBO TEK LIMITED</t>
+        </is>
+      </c>
+      <c r="C12" s="93" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D12" s="93" t="n">
+        <v>1513</v>
+      </c>
+      <c r="E12" s="93" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="F12" s="93" t="n">
+        <v>142805</v>
+      </c>
+      <c r="G12" s="93" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="H12" s="93" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I12" s="93" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J12" s="93" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="K12" s="93" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="L12" s="93" t="n">
+        <v>7</v>
+      </c>
+      <c r="M12" s="93" t="inlineStr">
+        <is>
+          <t>STRONG SETUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="91" t="inlineStr">
+        <is>
+          <t>RKFORGE</t>
+        </is>
+      </c>
+      <c r="B13" s="91" t="inlineStr">
+        <is>
+          <t>RAMKRISHNA FORGINGS LTD.</t>
+        </is>
+      </c>
+      <c r="C13" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D13" s="91" t="n">
+        <v>613.95</v>
+      </c>
+      <c r="E13" s="91" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="F13" s="91" t="n">
+        <v>6415288</v>
+      </c>
+      <c r="G13" s="91" t="n">
+        <v>393.87</v>
+      </c>
+      <c r="H13" s="91" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="I13" s="91" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="J13" s="91" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="K13" s="91" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="L13" s="91" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" s="91" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="93" t="inlineStr">
+        <is>
+          <t>KANSAINER</t>
+        </is>
+      </c>
+      <c r="B14" s="93" t="inlineStr">
+        <is>
+          <t>KANSAI NEROLAC PAINTS LTD.</t>
+        </is>
+      </c>
+      <c r="C14" s="93" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D14" s="93" t="n">
+        <v>204.12</v>
+      </c>
+      <c r="E14" s="93" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="F14" s="93" t="n">
+        <v>315111</v>
+      </c>
+      <c r="G14" s="93" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="H14" s="93" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="I14" s="93" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J14" s="93" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="K14" s="93" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="L14" s="93" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="93" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="91" t="inlineStr">
+        <is>
+          <t>PVRINOX</t>
+        </is>
+      </c>
+      <c r="B15" s="91" t="inlineStr">
+        <is>
+          <t>PVR INOX LIMITED</t>
+        </is>
+      </c>
+      <c r="C15" s="91" t="inlineStr">
+        <is>
+          <t>BSE Smallcap</t>
+        </is>
+      </c>
+      <c r="D15" s="91" t="n">
+        <v>1121.45</v>
+      </c>
+      <c r="E15" s="91" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F15" s="91" t="n">
+        <v>1056369</v>
+      </c>
+      <c r="G15" s="91" t="n">
+        <v>118.47</v>
+      </c>
+      <c r="H15" s="91" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I15" s="91" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J15" s="91" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="K15" s="91" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="L15" s="91" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="91" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="89" t="inlineStr">
+        <is>
+          <t>BSE SMALLCAP GAINERS — DEEP DIVE + LIKELY REASON — 11 stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1" s="45">
+      <c r="A18" s="90" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B18" s="90" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C18" s="90" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="D18" s="90" t="inlineStr">
+        <is>
+          <t>% Chg</t>
+        </is>
+      </c>
+      <c r="E18" s="90" t="inlineStr">
+        <is>
+          <t>Turnover (Rs Cr)</t>
+        </is>
+      </c>
+      <c r="F18" s="90" t="inlineStr">
+        <is>
+          <t>Vol Ratio (vs 3d avg)</t>
+        </is>
+      </c>
+      <c r="G18" s="90" t="inlineStr">
+        <is>
+          <t>Vol Ratio (vs 20d avg)</t>
+        </is>
+      </c>
+      <c r="H18" s="90" t="inlineStr">
+        <is>
+          <t>Trend Strength</t>
+        </is>
+      </c>
+      <c r="I18" s="90" t="inlineStr">
+        <is>
+          <t>20d Slope %/day</t>
+        </is>
+      </c>
+      <c r="J18" s="90" t="inlineStr">
+        <is>
+          <t>Trend R^2</t>
+        </is>
+      </c>
+      <c r="K18" s="90" t="inlineStr">
+        <is>
+          <t>Trend Quality (ADX x R^2)</t>
+        </is>
+      </c>
+      <c r="L18" s="90" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="M18" s="90" t="inlineStr">
+        <is>
+          <t>Stop Loss</t>
+        </is>
+      </c>
+      <c r="N18" s="90" t="inlineStr">
+        <is>
+          <t>Target 1</t>
+        </is>
+      </c>
+      <c r="O18" s="90" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="P18" s="90" t="inlineStr">
+        <is>
+          <t>Likely Reason for Gain</t>
+        </is>
+      </c>
+      <c r="Q18" s="90" t="inlineStr">
+        <is>
+          <t>Recent Headlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="95" t="inlineStr">
+        <is>
+          <t>KFINTECH</t>
+        </is>
+      </c>
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>KFin Technologies Limited</t>
+        </is>
+      </c>
+      <c r="C19" s="95" t="n">
+        <v>930.2</v>
+      </c>
+      <c r="D19" s="95" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="E19" s="95" t="n">
+        <v>426.42</v>
+      </c>
+      <c r="F19" s="95" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="G19" s="95" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H19" s="95" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I19" s="95" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="J19" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K19" s="95" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="L19" s="95" t="n">
+        <v>930.2</v>
+      </c>
+      <c r="M19" s="95" t="n">
+        <v>882.75</v>
+      </c>
+      <c r="N19" s="95" t="n">
+        <v>977.65</v>
+      </c>
+      <c r="O19" s="95" t="n">
+        <v>1025.11</v>
+      </c>
+      <c r="P19" s="95" t="inlineStr">
+        <is>
+          <t>Results / Earnings / Buyback</t>
+        </is>
+      </c>
+      <c r="Q19" s="95" t="inlineStr">
+        <is>
+          <t>KFin Tech Q1 Consolidated Net Profit Slides to 752M Rupees from 811M QoQ - Sahi; UltraTech sets Aug 17 for AGM, opens remote voting on Aug 13 - scanx.trade; Gabriel India schedules 64th AGM for August 19 with e-voting - scanx.trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="96" t="inlineStr">
+        <is>
+          <t>SAGILITY</t>
+        </is>
+      </c>
+      <c r="B20" s="96" t="inlineStr">
+        <is>
+          <t>Sagility Limited</t>
+        </is>
+      </c>
+      <c r="C20" s="96" t="n">
+        <v>43.37</v>
+      </c>
+      <c r="D20" s="96" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E20" s="96" t="n">
+        <v>283.49</v>
+      </c>
+      <c r="F20" s="96" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="G20" s="96" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="H20" s="96" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I20" s="96" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="J20" s="96" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K20" s="96" t="n">
+        <v>11</v>
+      </c>
+      <c r="L20" s="96" t="n">
+        <v>43.37</v>
+      </c>
+      <c r="M20" s="96" t="n">
+        <v>41.06</v>
+      </c>
+      <c r="N20" s="96" t="n">
+        <v>45.68</v>
+      </c>
+      <c r="O20" s="96" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="P20" s="96" t="inlineStr">
+        <is>
+          <t>No recent headlines found — verify BSE announcements manually; may be a pure technical/momentum breakout</t>
+        </is>
+      </c>
+      <c r="Q20" s="96" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="95" t="inlineStr">
+        <is>
+          <t>REDINGTON</t>
+        </is>
+      </c>
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Redington Limited</t>
+        </is>
+      </c>
+      <c r="C21" s="95" t="n">
+        <v>277.8</v>
+      </c>
+      <c r="D21" s="95" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="E21" s="95" t="n">
+        <v>109.65</v>
+      </c>
+      <c r="F21" s="95" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G21" s="95" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="H21" s="95" t="inlineStr">
+        <is>
+          <t>Weak / Range-bound</t>
+        </is>
+      </c>
+      <c r="I21" s="95" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="J21" s="95" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K21" s="95" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L21" s="95" t="n">
+        <v>277.8</v>
+      </c>
+      <c r="M21" s="95" t="n">
+        <v>292.05</v>
+      </c>
+      <c r="N21" s="95" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="O21" s="95" t="n">
+        <v>249.3</v>
+      </c>
+      <c r="P21" s="95" t="inlineStr">
+        <is>
+          <t>No recent headlines found — verify BSE announcements manually; may be a pure technical/momentum breakout</t>
+        </is>
+      </c>
+      <c r="Q21" s="95" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="96" t="inlineStr">
+        <is>
+          <t>LATENTVIEW</t>
+        </is>
+      </c>
+      <c r="B22" s="96" t="inlineStr">
+        <is>
+          <t>Latent View Analytics Limited</t>
+        </is>
+      </c>
+      <c r="C22" s="96" t="n">
+        <v>316.3</v>
+      </c>
+      <c r="D22" s="96" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="E22" s="96" t="n">
+        <v>112.53</v>
+      </c>
+      <c r="F22" s="96" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G22" s="96" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="H22" s="96" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I22" s="96" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J22" s="96" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K22" s="96" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="L22" s="96" t="n">
+        <v>316.3</v>
+      </c>
+      <c r="M22" s="96" t="n">
+        <v>298.88</v>
+      </c>
+      <c r="N22" s="96" t="n">
+        <v>333.72</v>
+      </c>
+      <c r="O22" s="96" t="n">
+        <v>351.13</v>
+      </c>
+      <c r="P22" s="96" t="inlineStr">
+        <is>
+          <t>No recent headlines found — verify BSE announcements manually; may be a pure technical/momentum breakout</t>
+        </is>
+      </c>
+      <c r="Q22" s="96" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="95" t="inlineStr">
+        <is>
+          <t>CAPLIPOINT</t>
+        </is>
+      </c>
+      <c r="B23" s="95" t="inlineStr">
+        <is>
+          <t>CAPLIN POINT LABORATORIES LTD.</t>
+        </is>
+      </c>
+      <c r="C23" s="95" t="n">
+        <v>2620.5</v>
+      </c>
+      <c r="D23" s="95" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E23" s="95" t="n">
+        <v>63.22</v>
+      </c>
+      <c r="F23" s="95" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="G23" s="95" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H23" s="95" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I23" s="95" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J23" s="95" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K23" s="95" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L23" s="95" t="n">
+        <v>2620.5</v>
+      </c>
+      <c r="M23" s="95" t="n">
+        <v>2770.26</v>
+      </c>
+      <c r="N23" s="95" t="n">
+        <v>2470.74</v>
+      </c>
+      <c r="O23" s="95" t="n">
+        <v>2320.97</v>
+      </c>
+      <c r="P23" s="95" t="inlineStr">
+        <is>
+          <t>No obvious corporate-action keyword in headlines — likely technical/momentum move; verify manually</t>
+        </is>
+      </c>
+      <c r="Q23" s="95" t="inlineStr">
+        <is>
+          <t>Top 14 Pharma Stocks To Buy In India July 2026 - Samco</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="96" t="inlineStr">
+        <is>
+          <t>LALPATHLAB</t>
+        </is>
+      </c>
+      <c r="B24" s="96" t="inlineStr">
+        <is>
+          <t>Dr. Lal Pathlabs Limited</t>
+        </is>
+      </c>
+      <c r="C24" s="96" t="n">
+        <v>1867.3</v>
+      </c>
+      <c r="D24" s="96" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="E24" s="96" t="n">
+        <v>315.37</v>
+      </c>
+      <c r="F24" s="96" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="G24" s="96" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="H24" s="96" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I24" s="96" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="J24" s="96" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="K24" s="96" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="L24" s="96" t="n">
+        <v>1867.3</v>
+      </c>
+      <c r="M24" s="96" t="n">
+        <v>1777.75</v>
+      </c>
+      <c r="N24" s="96" t="n">
+        <v>1956.85</v>
+      </c>
+      <c r="O24" s="96" t="n">
+        <v>2046.4</v>
+      </c>
+      <c r="P24" s="96" t="inlineStr">
+        <is>
+          <t>Dividend / Bonus / Split / Results / Earnings / Stake Sale / M&amp;A</t>
+        </is>
+      </c>
+      <c r="Q24" s="96" t="inlineStr">
+        <is>
+          <t>Dr. Lal PathLabs Independent Director Gurinder Singh Kalra steps down - scanx.trade; Dr Lal Pathlabs declares ₹4 final dividend per share at AGM - scanx.trade; Dr. Lal PathLabs Q1FY27 profit surges 27% to ₹1,705 Cr on revenue growth - scanx.trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="95" t="inlineStr">
+        <is>
+          <t>ATUL</t>
+        </is>
+      </c>
+      <c r="B25" s="95" t="inlineStr">
+        <is>
+          <t>ATUL LTD.</t>
+        </is>
+      </c>
+      <c r="C25" s="95" t="n">
+        <v>6799.5</v>
+      </c>
+      <c r="D25" s="95" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="E25" s="95" t="n">
+        <v>162.54</v>
+      </c>
+      <c r="F25" s="95" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G25" s="95" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="H25" s="95" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I25" s="95" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="J25" s="95" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="K25" s="95" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L25" s="95" t="n">
+        <v>6799.5</v>
+      </c>
+      <c r="M25" s="95" t="n">
+        <v>7118.23</v>
+      </c>
+      <c r="N25" s="95" t="n">
+        <v>6480.77</v>
+      </c>
+      <c r="O25" s="95" t="n">
+        <v>6162.04</v>
+      </c>
+      <c r="P25" s="95" t="inlineStr">
+        <is>
+          <t>Results / Earnings</t>
+        </is>
+      </c>
+      <c r="Q25" s="95" t="inlineStr">
+        <is>
+          <t>Atul Shares Extend Gains, Rise 4% After Sharp Improvement In Q1 Performance - NDTV Profit; Atul Ltd Q1 Results: Consolidated net profit surges 92% YoY - scanx.trade; Atul Ltd Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="96" t="inlineStr">
+        <is>
+          <t>TBOTEK</t>
+        </is>
+      </c>
+      <c r="B26" s="96" t="inlineStr">
+        <is>
+          <t>TBO TEK LIMITED</t>
+        </is>
+      </c>
+      <c r="C26" s="96" t="n">
+        <v>1513</v>
+      </c>
+      <c r="D26" s="96" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="E26" s="96" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="F26" s="96" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G26" s="96" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H26" s="96" t="inlineStr">
+        <is>
+          <t>Weak / Range-bound</t>
+        </is>
+      </c>
+      <c r="I26" s="96" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="J26" s="96" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="K26" s="96" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L26" s="96" t="n">
+        <v>1513</v>
+      </c>
+      <c r="M26" s="96" t="n">
+        <v>1583.29</v>
+      </c>
+      <c r="N26" s="96" t="n">
+        <v>1442.71</v>
+      </c>
+      <c r="O26" s="96" t="n">
+        <v>1372.43</v>
+      </c>
+      <c r="P26" s="96" t="inlineStr">
+        <is>
+          <t>No obvious corporate-action keyword in headlines — likely technical/momentum move; verify manually</t>
+        </is>
+      </c>
+      <c r="Q26" s="96" t="inlineStr">
+        <is>
+          <t>MEESHO LIMITED Share Price - Upstox</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="95" t="inlineStr">
+        <is>
+          <t>RKFORGE</t>
+        </is>
+      </c>
+      <c r="B27" s="95" t="inlineStr">
+        <is>
+          <t>RAMKRISHNA FORGINGS LTD.</t>
+        </is>
+      </c>
+      <c r="C27" s="95" t="n">
+        <v>613.95</v>
+      </c>
+      <c r="D27" s="95" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="E27" s="95" t="n">
+        <v>393.87</v>
+      </c>
+      <c r="F27" s="95" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G27" s="95" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H27" s="95" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I27" s="95" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J27" s="95" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K27" s="95" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="L27" s="95" t="n">
+        <v>613.95</v>
+      </c>
+      <c r="M27" s="95" t="n">
+        <v>584.08</v>
+      </c>
+      <c r="N27" s="95" t="n">
+        <v>643.8200000000001</v>
+      </c>
+      <c r="O27" s="95" t="n">
+        <v>673.6799999999999</v>
+      </c>
+      <c r="P27" s="95" t="inlineStr">
+        <is>
+          <t>Results / Earnings</t>
+        </is>
+      </c>
+      <c r="Q27" s="95" t="inlineStr">
+        <is>
+          <t>Earnings call transcript: Ramkrishna Forgings posts strong Q1 2027 growth - Investing.com; Ramkrishna Forgings Q1 FY27 slides: profit surges 297% on diversification By Investing.com; Ramkrishna Forgings Ltd Surges 7.38% to Day's High of Rs 614.9 — Outperforms Sector by 4.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="96" t="inlineStr">
+        <is>
+          <t>KANSAINER</t>
+        </is>
+      </c>
+      <c r="B28" s="96" t="inlineStr">
+        <is>
+          <t>KANSAI NEROLAC PAINTS LTD.</t>
+        </is>
+      </c>
+      <c r="C28" s="96" t="n">
+        <v>204.12</v>
+      </c>
+      <c r="D28" s="96" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="E28" s="96" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="F28" s="96" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="G28" s="96" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="H28" s="96" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="I28" s="96" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="J28" s="96" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="K28" s="96" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="L28" s="96" t="n">
+        <v>204.12</v>
+      </c>
+      <c r="M28" s="96" t="n">
+        <v>212.35</v>
+      </c>
+      <c r="N28" s="96" t="n">
+        <v>195.88</v>
+      </c>
+      <c r="O28" s="96" t="n">
+        <v>187.65</v>
+      </c>
+      <c r="P28" s="96" t="inlineStr">
+        <is>
+          <t>No recent headlines found — verify BSE announcements manually; may be a pure technical/momentum breakout</t>
+        </is>
+      </c>
+      <c r="Q28" s="96" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="95" t="inlineStr">
+        <is>
+          <t>PVRINOX</t>
+        </is>
+      </c>
+      <c r="B29" s="95" t="inlineStr">
+        <is>
+          <t>PVR INOX LIMITED</t>
+        </is>
+      </c>
+      <c r="C29" s="95" t="n">
+        <v>1121.45</v>
+      </c>
+      <c r="D29" s="95" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E29" s="95" t="n">
+        <v>118.47</v>
+      </c>
+      <c r="F29" s="95" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G29" s="95" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="H29" s="95" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I29" s="95" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J29" s="95" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="K29" s="95" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="L29" s="95" t="n">
+        <v>1121.45</v>
+      </c>
+      <c r="M29" s="95" t="n">
+        <v>1071.18</v>
+      </c>
+      <c r="N29" s="95" t="n">
+        <v>1171.72</v>
+      </c>
+      <c r="O29" s="95" t="n">
+        <v>1221.98</v>
+      </c>
+      <c r="P29" s="95" t="inlineStr">
+        <is>
+          <t>No obvious corporate-action keyword in headlines — likely technical/momentum move; verify manually</t>
+        </is>
+      </c>
+      <c r="Q29" s="95" t="inlineStr">
+        <is>
+          <t>Earnings call transcript: PVR INOX beats Q1 2026 EPS forecast as stock rises 4.8% - Invest; PVR INOX bets on sports, concerts and comedy to drive out-of-home entertainment growth - I; PVR INOX Diversifies Into Live Sports, Concerts To Boost Revenue - Whalesbook</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>